<commit_message>
iconicity english done !!
</commit_message>
<xml_diff>
--- a/iconicity_english/output/correlations.xlsx
+++ b/iconicity_english/output/correlations.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,7 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>openAI_4o</t>
+          <t>iconicity_english_base_prompt_gpt-4o</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>iconicity_english_base_prompt_gpt-4o_finetuned</t>
         </is>
       </c>
     </row>
@@ -433,14 +438,31 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>0.6193300732577068</v>
+        <v>0.6193300732577071</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.7614751677305192</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.6193300732577068</v>
+        <v>0.6193300732577071</v>
       </c>
       <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.801650714134854</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>0.7614751677305192</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.801650714134854</v>
+      </c>
+      <c r="C4" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>